<commit_message>
Update approved jobs sheet
</commit_message>
<xml_diff>
--- a/approved_jobs.xlsx
+++ b/approved_jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H466"/>
+  <dimension ref="A1:H465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -15911,17 +15911,17 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:56.748107+00:00</t>
+          <t>2026-08-22T12:32:54.751872+00:00</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Software Engineer Intern</t>
+          <t>Software Engineering Intern</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>FRND</t>
+          <t>Harman</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
@@ -15933,7 +15933,7 @@
       <c r="F412" t="inlineStr"/>
       <c r="G412" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4455599485/</t>
+          <t>https://jobsearch.harman.com/en_US/careers/searchjobs/R-54623-2026</t>
         </is>
       </c>
       <c r="H412" t="inlineStr">
@@ -15945,29 +15945,33 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:54.751872+00:00</t>
+          <t>2026-08-22T12:32:52.811769+00:00</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>Software Engineering Intern</t>
+          <t>AI Facial Data Collection Contributor</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Harman</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E413" t="inlineStr"/>
-      <c r="F413" t="inlineStr"/>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Remote (Work From Home)</t>
+        </is>
+      </c>
       <c r="G413" t="inlineStr">
         <is>
-          <t>https://jobsearch.harman.com/en_US/careers/searchjobs/R-54623-2026</t>
+          <t>https://bit.ly/4hl4Ar1</t>
         </is>
       </c>
       <c r="H413" t="inlineStr">
@@ -15979,12 +15983,12 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:52.811769+00:00</t>
+          <t>2026-08-22T12:32:50.619505+00:00</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>AI Facial Data Collection Contributor</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -15994,7 +15998,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E414" t="inlineStr"/>
@@ -16005,7 +16009,7 @@
       </c>
       <c r="G414" t="inlineStr">
         <is>
-          <t>https://bit.ly/4hl4Ar1</t>
+          <t>https://bit.ly/4hH3q9A</t>
         </is>
       </c>
       <c r="H414" t="inlineStr">
@@ -16017,17 +16021,17 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:50.619505+00:00</t>
+          <t>2026-08-22T12:32:48.755864+00:00</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Software Engineer - AMTS</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
@@ -16038,12 +16042,12 @@
       <c r="E415" t="inlineStr"/>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Remote (Work From Home)</t>
+          <t>Hyderabad/Bangalore, India</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
         <is>
-          <t>https://bit.ly/4hH3q9A</t>
+          <t>https://bit.ly/4xGBIOS</t>
         </is>
       </c>
       <c r="H415" t="inlineStr">
@@ -16055,33 +16059,33 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:48.755864+00:00</t>
+          <t>2026-08-22T12:32:43.264285+00:00</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Software Engineer - AMTS</t>
+          <t>Fullstack Developer</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>micro1</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="E416" t="inlineStr"/>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Hyderabad/Bangalore, India</t>
+          <t>Remote (Work From Home)</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
         <is>
-          <t>https://bit.ly/4xGBIOS</t>
+          <t>https://bit.ly/3Sy7PRO</t>
         </is>
       </c>
       <c r="H416" t="inlineStr">
@@ -16093,12 +16097,12 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:43.264285+00:00</t>
+          <t>2026-08-22T12:32:40.571545+00:00</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Fullstack Developer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -16108,7 +16112,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E417" t="inlineStr"/>
@@ -16119,7 +16123,7 @@
       </c>
       <c r="G417" t="inlineStr">
         <is>
-          <t>https://bit.ly/3Sy7PRO</t>
+          <t>https://bit.ly/4wZ8B9r</t>
         </is>
       </c>
       <c r="H417" t="inlineStr">
@@ -16131,50 +16135,50 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>2026-08-22T12:32:40.571545+00:00</t>
+          <t>2026-08-21T18:33:37.259219+00:00</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Intern - AI/ML</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E418" t="inlineStr"/>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Remote (Work From Home)</t>
+          <t>gurgaon</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
         <is>
-          <t>https://bit.ly/4wZ8B9r</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8143756</t>
         </is>
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>Found via Telegram channel @jobs_and_internships_updates. Verify details before approving.</t>
+          <t>Intern - AI/ML</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>2026-08-21T18:33:37.259219+00:00</t>
+          <t>2026-08-21T18:33:33.878834+00:00</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Intern - AI/ML</t>
+          <t>Quantitative Developer Intern</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -16184,226 +16188,222 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E419" t="inlineStr"/>
       <c r="F419" t="inlineStr">
         <is>
-          <t>gurgaon</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8143756</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8138524</t>
         </is>
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>Intern - AI/ML</t>
+          <t>Quantitative Developer Intern</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>2026-08-21T18:33:33.878834+00:00</t>
+          <t>2026-08-21T18:33:29.313779+00:00</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Quantitative Developer Intern</t>
+          <t>Sales &amp; Customer Success Intern - EU</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Truecaller</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E420" t="inlineStr"/>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8138524</t>
+          <t>https://job-boards.greenhouse.io/truecaller/jobs/8138837</t>
         </is>
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>Quantitative Developer Intern</t>
+          <t>Sales &amp; Customer Success Intern - EU</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>2026-08-21T18:33:29.313779+00:00</t>
+          <t>2026-08-14T03:46:04.307219+00:00</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Sales &amp; Customer Success Intern - EU</t>
+          <t>Quantitative Research Internship - 6 Months, Central Execution Research</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Truecaller</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E421" t="inlineStr"/>
       <c r="F421" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>London</t>
         </is>
       </c>
       <c r="G421" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/truecaller/jobs/8138837</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8113986</t>
         </is>
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t>Sales &amp; Customer Success Intern - EU</t>
+          <t>Quantitative Research Internship - 6 Months, Central Execution Research</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>2026-08-14T03:46:04.307219+00:00</t>
+          <t>2026-08-10T17:40:47.009978+00:00</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Quantitative Research Internship - 6 Months, Central Execution Research</t>
+          <t>[Backend] Software Engineering Intern</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Enterpret</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E422" t="inlineStr"/>
       <c r="F422" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Bengaluru, Onsite</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8113986</t>
+          <t>https://job-boards.greenhouse.io/enterpret/jobs/7847134003</t>
         </is>
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t>Quantitative Research Internship - 6 Months, Central Execution Research</t>
+          <t>[Backend] Software Engineering Intern</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>2026-08-10T17:40:47.009978+00:00</t>
+          <t>2026-08-08T04:12:52.37725+00:00</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>[Backend] Software Engineering Intern</t>
+          <t>Brand Marketing Intern</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Enterpret</t>
+          <t>Earnin</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E423" t="inlineStr"/>
-      <c r="F423" t="inlineStr">
-        <is>
-          <t>Bengaluru, Onsite</t>
-        </is>
-      </c>
+      <c r="F423" t="inlineStr"/>
       <c r="G423" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/enterpret/jobs/7847134003</t>
+          <t>https://job-boards.greenhouse.io/earnin/jobs/8113206</t>
         </is>
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t>[Backend] Software Engineering Intern</t>
+          <t>Brand Marketing Intern</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>2026-08-08T04:12:52.37725+00:00</t>
+          <t>2026-08-08T04:12:50.084908+00:00</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Brand Marketing Intern</t>
+          <t>Customer Success Intern</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Earnin</t>
+          <t>Knowbe4</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E424" t="inlineStr"/>
       <c r="F424" t="inlineStr"/>
       <c r="G424" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/earnin/jobs/8113206</t>
+          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8660687002</t>
         </is>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t>Brand Marketing Intern</t>
+          <t>Customer Success Intern</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>2026-08-08T04:12:50.084908+00:00</t>
+          <t>2026-08-08T04:12:45.117452+00:00</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Customer Success Intern</t>
+          <t>Junior Execution Trader Intern</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Knowbe4</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
@@ -16415,29 +16415,29 @@
       <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8660687002</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8091833</t>
         </is>
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>Customer Success Intern</t>
+          <t>Junior Execution Trader Intern</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>2026-08-08T04:12:45.117452+00:00</t>
+          <t>2026-07-27T16:30:43.226773+00:00</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Junior Execution Trader Intern</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
@@ -16449,24 +16449,24 @@
       <c r="F426" t="inlineStr"/>
       <c r="G426" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8091833</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
         </is>
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>Junior Execution Trader Intern</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:43.226773+00:00</t>
+          <t>2026-07-27T16:30:36.983937+00:00</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -16483,24 +16483,24 @@
       <c r="F427" t="inlineStr"/>
       <c r="G427" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
         </is>
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:36.983937+00:00</t>
+          <t>2026-07-27T16:30:35.138664+00:00</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t xml:space="preserve">Internship - Content </t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -16510,31 +16510,31 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E428" t="inlineStr"/>
       <c r="F428" t="inlineStr"/>
       <c r="G428" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
         </is>
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Internship - Content</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:35.138664+00:00</t>
+          <t>2026-07-27T16:30:33.590227+00:00</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internship - Content </t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -16544,65 +16544,65 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E429" t="inlineStr"/>
       <c r="F429" t="inlineStr"/>
       <c r="G429" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
         </is>
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>Internship - Content</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:33.590227+00:00</t>
+          <t>2026-07-27T16:30:31.543915+00:00</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Business Development Specialist (Outbound- International)</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Tide</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E430" t="inlineStr"/>
       <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
+          <t>https://job-boards.greenhouse.io/tide/jobs/7081017003</t>
         </is>
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Business Development Specialist (Outbound- International)</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:31.543915+00:00</t>
+          <t>2026-07-27T16:30:28.879852+00:00</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>Business Development Specialist (Outbound- International)</t>
+          <t>Business Development Specialist (International Sales)</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -16612,65 +16612,65 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E431" t="inlineStr"/>
       <c r="F431" t="inlineStr"/>
       <c r="G431" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/tide/jobs/7081017003</t>
+          <t>https://job-boards.greenhouse.io/tide/jobs/7598880003</t>
         </is>
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t>Business Development Specialist (Outbound- International)</t>
+          <t>Business Development Specialist (International Sales)</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:28.879852+00:00</t>
+          <t>2026-07-27T16:30:17.721593+00:00</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>Business Development Specialist (International Sales)</t>
+          <t>Risk Intern - 6 Month Internship Opportunity</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>Tide</t>
+          <t>Towerresearchcapital</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E432" t="inlineStr"/>
       <c r="F432" t="inlineStr"/>
       <c r="G432" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/tide/jobs/7598880003</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=7789933</t>
         </is>
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>Business Development Specialist (International Sales)</t>
+          <t>Risk Intern - 6 Month Internship Opportunity</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:17.721593+00:00</t>
+          <t>2026-07-27T16:30:10.248679+00:00</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>Risk Intern - 6 Month Internship Opportunity</t>
+          <t>Quantitative Trader Intern - Summer 2027</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -16687,24 +16687,24 @@
       <c r="F433" t="inlineStr"/>
       <c r="G433" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=7789933</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8024128</t>
         </is>
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>Risk Intern - 6 Month Internship Opportunity</t>
+          <t>Quantitative Trader Intern - Summer 2027</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:10.248679+00:00</t>
+          <t>2026-07-27T16:30:07.980596+00:00</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>Quantitative Trader Intern - Summer 2027</t>
+          <t>Quantitative Trader Intern, PhD</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -16721,24 +16721,24 @@
       <c r="F434" t="inlineStr"/>
       <c r="G434" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8024128</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8024138</t>
         </is>
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>Quantitative Trader Intern - Summer 2027</t>
+          <t>Quantitative Trader Intern, PhD</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:07.980596+00:00</t>
+          <t>2026-07-27T16:30:05.838281+00:00</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Quantitative Trader Intern, PhD</t>
+          <t>Quantitative Developer Intern - Summer 2027</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
@@ -16755,24 +16755,24 @@
       <c r="F435" t="inlineStr"/>
       <c r="G435" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8024138</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8044334</t>
         </is>
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t>Quantitative Trader Intern, PhD</t>
+          <t>Quantitative Developer Intern - Summer 2027</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:05.838281+00:00</t>
+          <t>2026-07-27T16:30:03.426202+00:00</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>Quantitative Developer Intern - Summer 2027</t>
+          <t>Business Analytics Intern - 6 Month Internship Opportunity</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
@@ -16782,60 +16782,60 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E436" t="inlineStr"/>
       <c r="F436" t="inlineStr"/>
       <c r="G436" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8044334</t>
+          <t>https://www.tower-research.com/open-positions/?gh_jid=8041512</t>
         </is>
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t>Quantitative Developer Intern - Summer 2027</t>
+          <t>Business Analytics Intern - 6 Month Internship Opportunity</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:03.426202+00:00</t>
+          <t>2026-07-27T16:30:01.432263+00:00</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>Business Analytics Intern - 6 Month Internship Opportunity</t>
+          <t>Sales Development Representative Intern (Hybrid)</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Towerresearchcapital</t>
+          <t>Knowbe4</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E437" t="inlineStr"/>
       <c r="F437" t="inlineStr"/>
       <c r="G437" t="inlineStr">
         <is>
-          <t>https://www.tower-research.com/open-positions/?gh_jid=8041512</t>
+          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8566454002</t>
         </is>
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>Business Analytics Intern - 6 Month Internship Opportunity</t>
+          <t>Sales Development Representative Intern (Hybrid)</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>2026-07-27T16:30:01.432263+00:00</t>
+          <t>2026-07-27T16:29:59.490728+00:00</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
@@ -16857,7 +16857,7 @@
       <c r="F438" t="inlineStr"/>
       <c r="G438" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8566454002</t>
+          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8566457002</t>
         </is>
       </c>
       <c r="H438" t="inlineStr">
@@ -16869,41 +16869,41 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:59.490728+00:00</t>
+          <t>2026-07-27T16:29:55.183092+00:00</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>Sales Development Representative Intern (Hybrid)</t>
+          <t>Intern - Industrial Trainee</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Knowbe4</t>
+          <t>Inmobi</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E439" t="inlineStr"/>
       <c r="F439" t="inlineStr"/>
       <c r="G439" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/knowbe4/jobs/8566457002</t>
+          <t>https://job-boards.greenhouse.io/inmobi/jobs/8029868</t>
         </is>
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t>Sales Development Representative Intern (Hybrid)</t>
+          <t>Intern - Industrial Trainee</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:55.183092+00:00</t>
+          <t>2026-07-27T16:29:52.581754+00:00</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
@@ -16925,7 +16925,7 @@
       <c r="F440" t="inlineStr"/>
       <c r="G440" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/inmobi/jobs/8029868</t>
+          <t>https://job-boards.greenhouse.io/inmobi/jobs/7793050</t>
         </is>
       </c>
       <c r="H440" t="inlineStr">
@@ -16937,46 +16937,46 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:52.581754+00:00</t>
+          <t>2026-07-27T16:29:48.780995+00:00</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>Intern - Industrial Trainee</t>
+          <t>Security Consultant Intern</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Inmobi</t>
+          <t>Cloudsek</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Data / AI</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E441" t="inlineStr"/>
       <c r="F441" t="inlineStr"/>
       <c r="G441" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/inmobi/jobs/7793050</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6115382004</t>
         </is>
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t>Intern - Industrial Trainee</t>
+          <t>Security Consultant Intern</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:48.780995+00:00</t>
+          <t>2026-07-27T16:29:47.193044+00:00</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Security Consultant Intern</t>
+          <t xml:space="preserve">SDE Intern - Frontend   </t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -16986,31 +16986,31 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="E442" t="inlineStr"/>
       <c r="F442" t="inlineStr"/>
       <c r="G442" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6115382004</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/5831215004</t>
         </is>
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>Security Consultant Intern</t>
+          <t>SDE Intern - Frontend</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:47.193044+00:00</t>
+          <t>2026-07-27T16:29:44.845632+00:00</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t xml:space="preserve">SDE Intern - Frontend   </t>
+          <t>SDE - Backend - Intern</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -17020,31 +17020,31 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E443" t="inlineStr"/>
       <c r="F443" t="inlineStr"/>
       <c r="G443" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cloudsek/jobs/5831215004</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/5766402004</t>
         </is>
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t>SDE Intern - Frontend</t>
+          <t>SDE - Backend - Intern</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:44.845632+00:00</t>
+          <t>2026-07-27T16:29:42.382537+00:00</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>SDE - Backend - Intern</t>
+          <t>Business Development Representative Intern - Canada</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
@@ -17054,36 +17054,36 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E444" t="inlineStr"/>
       <c r="F444" t="inlineStr"/>
       <c r="G444" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cloudsek/jobs/5766402004</t>
+          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6005469004</t>
         </is>
       </c>
       <c r="H444" t="inlineStr">
         <is>
-          <t>SDE - Backend - Intern</t>
+          <t>Business Development Representative Intern - Canada</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:42.382537+00:00</t>
+          <t>2026-07-27T16:29:12.993097+00:00</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>Business Development Representative Intern - Canada</t>
+          <t>[Tech Cooperative Internship 2026] Software Engineer in Back End intern (6 months)</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Cloudsek</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
@@ -17095,24 +17095,24 @@
       <c r="F445" t="inlineStr"/>
       <c r="G445" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cloudsek/jobs/6005469004</t>
+          <t>https://job-boards.greenhouse.io/agoda/jobs/5443559</t>
         </is>
       </c>
       <c r="H445" t="inlineStr">
         <is>
-          <t>Business Development Representative Intern - Canada</t>
+          <t>[Tech Cooperative Internship 2026] Software Engineer in Back End intern (6 months)</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>2026-07-27T16:29:12.993097+00:00</t>
+          <t>2026-07-27T16:28:57.849831+00:00</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>[Tech Cooperative Internship 2026] Software Engineer in Back End intern (6 months)</t>
+          <t>International Payroll Partner</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -17129,29 +17129,29 @@
       <c r="F446" t="inlineStr"/>
       <c r="G446" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/agoda/jobs/5443559</t>
+          <t>https://job-boards.greenhouse.io/agoda/jobs/8063978</t>
         </is>
       </c>
       <c r="H446" t="inlineStr">
         <is>
-          <t>[Tech Cooperative Internship 2026] Software Engineer in Back End intern (6 months)</t>
+          <t>International Payroll Partner</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>2026-07-27T16:28:57.849831+00:00</t>
+          <t>2026-07-27T10:49:04.274532+00:00</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>International Payroll Partner</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="D447" t="inlineStr">
@@ -17163,24 +17163,24 @@
       <c r="F447" t="inlineStr"/>
       <c r="G447" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/agoda/jobs/8063978</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
         </is>
       </c>
       <c r="H447" t="inlineStr">
         <is>
-          <t>International Payroll Partner</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>2026-07-27T10:49:04.274532+00:00</t>
+          <t>2026-07-27T10:49:00.838626+00:00</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
@@ -17197,24 +17197,24 @@
       <c r="F448" t="inlineStr"/>
       <c r="G448" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
         </is>
       </c>
       <c r="H448" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>2026-07-27T10:49:00.838626+00:00</t>
+          <t>2026-07-27T10:48:58.630946+00:00</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t xml:space="preserve">Internship - Content </t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -17224,31 +17224,31 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E449" t="inlineStr"/>
       <c r="F449" t="inlineStr"/>
       <c r="G449" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
         </is>
       </c>
       <c r="H449" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Internship - Content</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>2026-07-27T10:48:58.630946+00:00</t>
+          <t>2026-07-27T10:48:56.06648+00:00</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internship - Content </t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -17258,31 +17258,31 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E450" t="inlineStr"/>
       <c r="F450" t="inlineStr"/>
       <c r="G450" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
         </is>
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t>Internship - Content</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>2026-07-27T10:48:56.06648+00:00</t>
+          <t>2026-07-27T10:42:53.996409+00:00</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -17292,31 +17292,31 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E451" t="inlineStr"/>
       <c r="F451" t="inlineStr"/>
       <c r="G451" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
         </is>
       </c>
       <c r="H451" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Copy Writer - Intern</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>2026-07-27T10:42:53.996409+00:00</t>
+          <t>2026-07-27T10:42:50.938109+00:00</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
@@ -17326,31 +17326,31 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E452" t="inlineStr"/>
       <c r="F452" t="inlineStr"/>
       <c r="G452" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774341101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
         </is>
       </c>
       <c r="H452" t="inlineStr">
         <is>
-          <t>Copy Writer - Intern</t>
+          <t>Graphic Designer - Intern</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>2026-07-27T10:42:50.938109+00:00</t>
+          <t>2026-07-27T10:42:47.32783+00:00</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t xml:space="preserve">Internship - Content </t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
@@ -17360,31 +17360,31 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E453" t="inlineStr"/>
       <c r="F453" t="inlineStr"/>
       <c r="G453" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4774342101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
         </is>
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>Graphic Designer - Intern</t>
+          <t>Internship - Content</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>2026-07-27T10:42:47.32783+00:00</t>
+          <t>2026-07-27T10:42:43.192382+00:00</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internship - Content </t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
@@ -17394,103 +17394,103 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E454" t="inlineStr"/>
       <c r="F454" t="inlineStr"/>
       <c r="G454" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4819749101</t>
+          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
         </is>
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t>Internship - Content</t>
+          <t>Video Editor Intern</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>2026-07-27T10:42:43.192382+00:00</t>
+          <t>2026-07-26T19:14:17.297621+00:00</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>ReactJS Internship</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>ElevateHQ</t>
         </is>
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="E455" t="inlineStr"/>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>₹240000 - ₹420000</t>
+        </is>
+      </c>
       <c r="F455" t="inlineStr"/>
       <c r="G455" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/groww/jobs/4771440101</t>
+          <t>https://www.adzuna.in/details/4794473734?utm_medium=api&amp;utm_source=e044e1cb</t>
         </is>
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t>Video Editor Intern</t>
+          <t>Position Overview: We are seeking a talented and motivated ReactJS Intern to join our team for a 6-month full-time internship. This is a fantastic opportunity for someone with prior internship experience to deepen their knowledge and skills in ReactJS while working on cutting-edge projects. Responsibilities: Collaborate with the development team to design, develop, and maintain web applications using ReactJS. Write clean, maintainable, and efficient code. Participate in code reviews and contrib…</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>2026-07-26T19:14:17.297621+00:00</t>
+          <t>2026-07-26T19:14:13.725695+00:00</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>ReactJS Internship</t>
+          <t>Developer Internship</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>ElevateHQ</t>
+          <t>PBL India</t>
         </is>
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="E456" t="inlineStr">
-        <is>
-          <t>₹240000 - ₹420000</t>
-        </is>
-      </c>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr"/>
       <c r="F456" t="inlineStr"/>
       <c r="G456" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/4794473734?utm_medium=api&amp;utm_source=e044e1cb</t>
+          <t>https://www.adzuna.in/details/4801600698?utm_medium=api&amp;utm_source=e044e1cb</t>
         </is>
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t>Position Overview: We are seeking a talented and motivated ReactJS Intern to join our team for a 6-month full-time internship. This is a fantastic opportunity for someone with prior internship experience to deepen their knowledge and skills in ReactJS while working on cutting-edge projects. Responsibilities: Collaborate with the development team to design, develop, and maintain web applications using ReactJS. Write clean, maintainable, and efficient code. Participate in code reviews and contrib…</t>
+          <t>Percpktika Brand Lab is a Product Development startup which supports and develops products guiding social innovation. We are looking for smart and talented interns who are capable of working from Delhi or remote and submitting results. At PBL we have an efficient training process which provides resources to grow and nurture your talent. The selected intern(s) will work on following during the internship: 1. Code Reviews and Research. 2. Creating Core features using Node.js and Native Script sup…</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>2026-07-26T19:14:13.725695+00:00</t>
+          <t>2026-07-26T19:14:07.63634+00:00</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>Developer Internship</t>
+          <t>Design Internship</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
@@ -17500,65 +17500,65 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E457" t="inlineStr"/>
       <c r="F457" t="inlineStr"/>
       <c r="G457" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/4801600698?utm_medium=api&amp;utm_source=e044e1cb</t>
+          <t>https://www.adzuna.in/details/4801437257?utm_medium=api&amp;utm_source=e044e1cb</t>
         </is>
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>Percpktika Brand Lab is a Product Development startup which supports and develops products guiding social innovation. We are looking for smart and talented interns who are capable of working from Delhi or remote and submitting results. At PBL we have an efficient training process which provides resources to grow and nurture your talent. The selected intern(s) will work on following during the internship: 1. Code Reviews and Research. 2. Creating Core features using Node.js and Native Script sup…</t>
+          <t>Percpktika Brand Lab is a Product Development startup which supports and develops products guiding social innovation. We are looking for smart and talented interns who are capable of working from Delhi or remote and submitting results. At PBL we have an efficient training process which provides resources to grow and nurture your talent. The selected intern(s) will work on following during the internship: 1. Designing User Interface. 2. Experience planning and flow. 3. Product Branding and Desig…</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>2026-07-26T19:14:07.63634+00:00</t>
+          <t>2026-07-26T19:13:19.489348+00:00</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>Design Internship</t>
+          <t>Customer Care Intern</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>PBL India</t>
+          <t>Criteo</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="E458" t="inlineStr"/>
       <c r="F458" t="inlineStr"/>
       <c r="G458" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/4801437257?utm_medium=api&amp;utm_source=e044e1cb</t>
+          <t>https://www.adzuna.in/land/ad/5790410523?se=rFvE0iWJ8RGGXqQIyNVN5Q&amp;utm_medium=api&amp;utm_source=e044e1cb&amp;v=5E72C4726A0DF728D03FF51102E0532CA986DDEA</t>
         </is>
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>Percpktika Brand Lab is a Product Development startup which supports and develops products guiding social innovation. We are looking for smart and talented interns who are capable of working from Delhi or remote and submitting results. At PBL we have an efficient training process which provides resources to grow and nurture your talent. The selected intern(s) will work on following during the internship: 1. Designing User Interface. 2. Experience planning and flow. 3. Product Branding and Desig…</t>
+          <t>This job is with Criteo, an inclusive employer and a member of myGwork – the largest global platform for the LGBTQ business community. Please do not contact the recruiter directly. What You'll Do: The multinational Global Customer Care Team is the first point of contact for Criteo Customers; our goal is to provide excellent customer support to all incoming client requests using email or live chat. We excel at collaboration, communication, and teamwork, as they are key to solving our client's re…</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>2026-07-26T19:13:19.489348+00:00</t>
+          <t>2026-07-26T19:13:17.765892+00:00</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>Customer Care Intern</t>
+          <t>Sales &amp; Strategy Intern</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -17568,259 +17568,225 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E459" t="inlineStr"/>
       <c r="F459" t="inlineStr"/>
       <c r="G459" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5790410523?se=rFvE0iWJ8RGGXqQIyNVN5Q&amp;utm_medium=api&amp;utm_source=e044e1cb&amp;v=5E72C4726A0DF728D03FF51102E0532CA986DDEA</t>
+          <t>https://www.adzuna.in/land/ad/5806276940?se=rFvE0iWJ8RGGXqQIyNVN5Q&amp;utm_medium=api&amp;utm_source=e044e1cb&amp;v=B2147145725F724ABD3B0362E330EB1DD5EB962B</t>
         </is>
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>This job is with Criteo, an inclusive employer and a member of myGwork – the largest global platform for the LGBTQ business community. Please do not contact the recruiter directly. What You'll Do: The multinational Global Customer Care Team is the first point of contact for Criteo Customers; our goal is to provide excellent customer support to all incoming client requests using email or live chat. We excel at collaboration, communication, and teamwork, as they are key to solving our client's re…</t>
+          <t>This job is with Criteo, an inclusive employer and a member of myGwork – the largest global platform for the LGBTQ business community. Please do not contact the recruiter directly. What You'll Do: As a Sales &amp; Strategy Intern, you will be part of our India team that works with new and existing clients. You will be learning and working with brands, analyzing and optimizing campaigns, along with cultivating a strong and productive relationship with clients. This is a 12-month paid, full-time inte…</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>2026-07-26T19:13:17.765892+00:00</t>
+          <t>2026-07-26T18:23:56.921677+00:00</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>Sales &amp; Strategy Intern</t>
+          <t>GRAPHIC DESIGNER</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Criteo</t>
+          <t>NEW VINE LIMITED</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E460" t="inlineStr"/>
       <c r="F460" t="inlineStr"/>
       <c r="G460" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5806276940?se=rFvE0iWJ8RGGXqQIyNVN5Q&amp;utm_medium=api&amp;utm_source=e044e1cb&amp;v=B2147145725F724ABD3B0362E330EB1DD5EB962B</t>
+          <t>https://remoteOK.com/remote-jobs/remote-graphic-designer-new-vine-limited-1135316</t>
         </is>
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>This job is with Criteo, an inclusive employer and a member of myGwork – the largest global platform for the LGBTQ business community. Please do not contact the recruiter directly. What You'll Do: As a Sales &amp; Strategy Intern, you will be part of our India team that works with new and existing clients. You will be learning and working with brands, analyzing and optimizing campaigns, along with cultivating a strong and productive relationship with clients. This is a 12-month paid, full-time inte…</t>
+          <t>Graphic Designer (part-time) An exciting opportunity has arisen for a Graphic Designer (part-time) to join us, working remotely with great benefits. The role will work primarily on our books, subscription materials, and digital resources, creating eye-catching covers, inside layouts, and ebooks. Prior experience of working on these types of resources in Adobe Creative Suite is essential, as is a solid understanding of design, layout, typography, and brand. Salary: Â£16,500 (Â£27,500 FTE) Applications close: 29 August 2026 Download the job information (.pdf) Download the application form (.docx) We welcome applicants from all backgrounds and communities, in particular those that are currently under-represented within our staff team. This includes, but is not limited to, people from Black, Asian, and other ethnic groups, especially within our leadership roles. Please mention the word **PROLIFIC** and tag RMjAyLjY2LjE2NC42 when applying to show you read the job post completely (#RMjAyLjY2LjE2NC42). This is a beta feature to avoid spam applicants. Companies can search these words to find applicants that read this and see they're human.</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:56.921677+00:00</t>
+          <t>2026-07-26T18:23:39.597545+00:00</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>GRAPHIC DESIGNER</t>
+          <t>Executive Assistant</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>NEW VINE LIMITED</t>
+          <t>Ritual AdsÂ®</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E461" t="inlineStr"/>
       <c r="F461" t="inlineStr"/>
       <c r="G461" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-graphic-designer-new-vine-limited-1135316</t>
+          <t>https://remoteOK.com/remote-jobs/remote-executive-assistant-ritual-adsr-1135344</t>
         </is>
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>Graphic Designer (part-time) An exciting opportunity has arisen for a Graphic Designer (part-time) to join us, working remotely with great benefits. The role will work primarily on our books, subscription materials, and digital resources, creating eye-catching covers, inside layouts, and ebooks. Prior experience of working on these types of resources in Adobe Creative Suite is essential, as is a solid understanding of design, layout, typography, and brand. Salary: Â£16,500 (Â£27,500 FTE) Applications close: 29 August 2026 Download the job information (.pdf) Download the application form (.docx) We welcome applicants from all backgrounds and communities, in particular those that are currently under-represented within our staff team. This includes, but is not limited to, people from Black, Asian, and other ethnic groups, especially within our leadership roles. Please mention the word **PROLIFIC** and tag RMjAyLjY2LjE2NC42 when applying to show you read the job post completely (#RMjAyLjY2LjE2NC42). This is a beta feature to avoid spam applicants. Companies can search these words to find applicants that read this and see they're human.</t>
+          <t>Company Description Ritual AdsÂ® is a cutting-edge AI software company that uses generative AI to create tailored, data-driven advertising content on demand. The platform helps organizations quickly produce high-impact, customized ads that align with their brand and audience. By combining advanced machine learning with real-time data, Ritual AdsÂ® aims to improve campaign performance and efficiency. Team members collaborate in a technology-forward environment focused on innovation, scalability, and measurable results. Role Description The Executive Assistant at Ritual AdsÂ® is a full-time, remote role responsible for providing comprehensive administrative and organizational support to company leadership. Day-to-day tasks include managing calendars, scheduling meetings, coordinating travel, and preparing agendas and meeting materials. The Executive Assistant will handle expense reports, track reimbursements, and maintain accurate documentation. The role also includes managing correspondence, drafting and editing communications, organizing digital files, and supporting special projects and operational tasks to ensure smooth executive workflows. Qualifications Strong Executive Adminis</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:39.597545+00:00</t>
+          <t>2026-07-26T18:23:35.307873+00:00</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>Executive Assistant</t>
+          <t>Product Designer</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>Ritual AdsÂ®</t>
+          <t>Flint</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E462" t="inlineStr"/>
       <c r="F462" t="inlineStr"/>
       <c r="G462" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-executive-assistant-ritual-adsr-1135344</t>
+          <t>https://remoteOK.com/remote-jobs/remote-product-designer-flint-1135340</t>
         </is>
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>Company Description Ritual AdsÂ® is a cutting-edge AI software company that uses generative AI to create tailored, data-driven advertising content on demand. The platform helps organizations quickly produce high-impact, customized ads that align with their brand and audience. By combining advanced machine learning with real-time data, Ritual AdsÂ® aims to improve campaign performance and efficiency. Team members collaborate in a technology-forward environment focused on innovation, scalability, and measurable results. Role Description The Executive Assistant at Ritual AdsÂ® is a full-time, remote role responsible for providing comprehensive administrative and organizational support to company leadership. Day-to-day tasks include managing calendars, scheduling meetings, coordinating travel, and preparing agendas and meeting materials. The Executive Assistant will handle expense reports, track reimbursements, and maintain accurate documentation. The role also includes managing correspondence, drafting and editing communications, organizing digital files, and supporting special projects and operational tasks to ensure smooth executive workflows. Qualifications Strong Executive Adminis</t>
+          <t>Compensation: $160kâ190k base + meaningful equity About Flint The best education anyone has ever received is one person paying close attention to one student: moving at their pace, noticing what they missed, asking the next question at the right moment. But the current system is built around a compromise with one teacher managing thirty students. Flint exists to take that compromise off the table. Personalized learning, at the scale of a whole school â every student working with something closer to a tutor, and every teacher able to see what's actually happening across their class instead of guessing. Go look at the product before you read any further: app.flintk12.com The Role Students want something that stays with them, going at their pace and helps them get unstuck without just handing over the answer. Teachers want that happening inside a class they still control, and they'd like their evenings back. Admins want proof that the platform they rolled out is leading to teacher productivity and student progress. Your job is to dive deep into this design problem, holding three sets of needs within one product. Weâll trust you to ship designs that are the best possible solution</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:35.307873+00:00</t>
+          <t>2026-07-26T18:23:18.030686+00:00</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>Product Designer</t>
+          <t>Join our UK team</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Workdry Germany</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E463" t="inlineStr"/>
       <c r="F463" t="inlineStr"/>
       <c r="G463" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-product-designer-flint-1135340</t>
+          <t>https://remoteOK.com/remote-jobs/remote-join-our-uk-team-workdry-germany-1135314</t>
         </is>
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>Compensation: $160kâ190k base + meaningful equity About Flint The best education anyone has ever received is one person paying close attention to one student: moving at their pace, noticing what they missed, asking the next question at the right moment. But the current system is built around a compromise with one teacher managing thirty students. Flint exists to take that compromise off the table. Personalized learning, at the scale of a whole school â every student working with something closer to a tutor, and every teacher able to see what's actually happening across their class instead of guessing. Go look at the product before you read any further: app.flintk12.com The Role Students want something that stays with them, going at their pace and helps them get unstuck without just handing over the answer. Teachers want that happening inside a class they still control, and they'd like their evenings back. Admins want proof that the platform they rolled out is leading to teacher productivity and student progress. Your job is to dive deep into this design problem, holding three sets of needs within one product. Weâll trust you to ship designs that are the best possible solution</t>
+          <t>BracknellPump Rental SolutionsBracknellPump Rental SolutionsGreat YarmouthPump Rental SolutionsNottinghamPump Rental SolutionsAberdeenPump Rental SolutionsConwyPump Rental SolutionsStokeWorkdry - Group Central ServicesStokeWorkdry - Group Central ServicesWorkingtonPump Rental Solutions Please mention the word **GREATNESS** and tag RMjAyLjY2LjE2NC42 when applying to show you read the job post completely (#RMjAyLjY2LjE2NC42). This is a beta feature to avoid spam applicants. Companies can search these words to find applicants that read this and see they're human.</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:18.030686+00:00</t>
+          <t>2026-07-26T18:23:11.834056+00:00</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>Join our UK team</t>
+          <t>Safety Data Analyst</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Workdry Germany</t>
+          <t>SkyWest Airlines</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Data / AI</t>
         </is>
       </c>
       <c r="E464" t="inlineStr"/>
       <c r="F464" t="inlineStr"/>
       <c r="G464" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-join-our-uk-team-workdry-germany-1135314</t>
+          <t>https://remoteOK.com/remote-jobs/remote-safety-data-analyst-skywest-airlines-1135445</t>
         </is>
       </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t>BracknellPump Rental SolutionsBracknellPump Rental SolutionsGreat YarmouthPump Rental SolutionsNottinghamPump Rental SolutionsAberdeenPump Rental SolutionsConwyPump Rental SolutionsStokeWorkdry - Group Central ServicesStokeWorkdry - Group Central ServicesWorkingtonPump Rental Solutions Please mention the word **GREATNESS** and tag RMjAyLjY2LjE2NC42 when applying to show you read the job post completely (#RMjAyLjY2LjE2NC42). This is a beta feature to avoid spam applicants. Companies can search these words to find applicants that read this and see they're human.</t>
+          <t>About SkyWest With over 16,000 aviation professionals operating thousands of daily flights, SkyWest Airlines connects millions of passengers each month to hundreds of destinations across North America. SkyWest operates in partnership with Delta Air Lines, United Airlines, American Airlines, and Alaska Airlines and has a fleet of nearly 450 aircraft. Headquartered in St. George, Utah, SkyWest's industry-leading workforce and excellent leadership team have consistently generated solid operational and economic performance, setting the standard for excellence in the regional industry. SkyWest employees enjoy a distinctive and unmatched culture of teamwork, respect, quality, and professionalism, along with world-class benefits such as a 401(k) match, Performance Rewards, health care, retirement, and discounted travel worldwide. Primary Job Duties Analyze, compile, and report safety data to support all SkyWest safety programs. Collect, analyze, and report safety assurance data from multiple safety data sources. Identify, monitor, and communicate safety performance trends and emerging risks. Track, maintain, and report key performance indicators (KPIs) for the Safety Department, including</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>2026-07-26T18:23:11.834056+00:00</t>
+          <t>2026-07-17T10:23:01.374271+00:00</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>Safety Data Analyst</t>
+          <t>Test Internship</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>SkyWest Airlines</t>
+          <t>Test Company</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>Data / AI</t>
-        </is>
-      </c>
-      <c r="E465" t="inlineStr"/>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>10,000/mo</t>
+        </is>
+      </c>
       <c r="F465" t="inlineStr"/>
       <c r="G465" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-safety-data-analyst-skywest-airlines-1135445</t>
+          <t>https://example.com</t>
         </is>
       </c>
       <c r="H465" t="inlineStr">
-        <is>
-          <t>About SkyWest With over 16,000 aviation professionals operating thousands of daily flights, SkyWest Airlines connects millions of passengers each month to hundreds of destinations across North America. SkyWest operates in partnership with Delta Air Lines, United Airlines, American Airlines, and Alaska Airlines and has a fleet of nearly 450 aircraft. Headquartered in St. George, Utah, SkyWest's industry-leading workforce and excellent leadership team have consistently generated solid operational and economic performance, setting the standard for excellence in the regional industry. SkyWest employees enjoy a distinctive and unmatched culture of teamwork, respect, quality, and professionalism, along with world-class benefits such as a 401(k) match, Performance Rewards, health care, retirement, and discounted travel worldwide. Primary Job Duties Analyze, compile, and report safety data to support all SkyWest safety programs. Collect, analyze, and report safety assurance data from multiple safety data sources. Identify, monitor, and communicate safety performance trends and emerging risks. Track, maintain, and report key performance indicators (KPIs) for the Safety Department, including</t>
-        </is>
-      </c>
-    </row>
-    <row r="466">
-      <c r="A466" t="inlineStr">
-        <is>
-          <t>2026-07-17T10:23:01.374271+00:00</t>
-        </is>
-      </c>
-      <c r="B466" t="inlineStr">
-        <is>
-          <t>Test Internship</t>
-        </is>
-      </c>
-      <c r="C466" t="inlineStr">
-        <is>
-          <t>Test Company</t>
-        </is>
-      </c>
-      <c r="D466" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="E466" t="inlineStr">
-        <is>
-          <t>10,000/mo</t>
-        </is>
-      </c>
-      <c r="F466" t="inlineStr"/>
-      <c r="G466" t="inlineStr">
-        <is>
-          <t>https://example.com</t>
-        </is>
-      </c>
-      <c r="H466" t="inlineStr">
         <is>
           <t>This is a test listing</t>
         </is>

</xml_diff>